<commit_message>
fix: clean PurchPurchaseOrder template + fix formula-as-text bug + auto-widen columns
- Clean PurchPurchaseOrder sheet (delete old data rows 33-51)
- Fix formula prefix bug: set cell.data_type='f' before writing formulas
- Auto-widen text columns (C, E) based on content length
- PPO cross-sheet refs use CONCATENATE for item descriptions
</commit_message>
<xml_diff>
--- a/stored_files/templates/DAINESE/DAINESE_VAN_CHUYEN_template.xlsx
+++ b/stored_files/templates/DAINESE/DAINESE_VAN_CHUYEN_template.xlsx
@@ -2700,7 +2700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB68"/>
+  <dimension ref="A1:AB48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="0.453125" customWidth="1" style="170" min="1" max="1"/>
@@ -3210,760 +3210,232 @@
       <c r="T32" s="181" t="inlineStr"/>
     </row>
     <row r="33" ht="17.5" customHeight="1">
-      <c r="A33" s="169" t="n">
-        <v>2</v>
-      </c>
-      <c r="C33" s="171" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cước vận chuyển KCN Yên Bình- Tam Dương </t>
-        </is>
-      </c>
-      <c r="F33" s="200">
-        <f>HĐ!H16</f>
-        <v/>
-      </c>
-      <c r="I33" s="174" t="n">
-        <v>1</v>
-      </c>
-      <c r="L33" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M33" s="267">
-        <f>HĐ!B16</f>
-        <v/>
-      </c>
-      <c r="P33" s="65">
-        <f>HĐ!N16</f>
-        <v/>
-      </c>
-      <c r="Q33" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" s="268">
-        <f>P33</f>
-        <v/>
-      </c>
-      <c r="T33" s="179" t="n"/>
-      <c r="Y33" s="171" t="n"/>
+      <c r="A33" s="199" t="n"/>
+      <c r="B33" s="261" t="n"/>
+      <c r="C33" s="199" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="D33" s="261" t="n"/>
+      <c r="E33" s="261" t="n"/>
+      <c r="F33" s="199" t="inlineStr">
+        <is>
+          <t>Subtotal Amount</t>
+        </is>
+      </c>
+      <c r="G33" s="261" t="n"/>
+      <c r="H33" s="261" t="n"/>
+      <c r="I33" s="197" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+      <c r="J33" s="261" t="n"/>
+      <c r="K33" s="261" t="n"/>
+      <c r="L33" s="197" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="M33" s="197" t="inlineStr">
+        <is>
+          <t>Sales tax</t>
+        </is>
+      </c>
+      <c r="N33" s="261" t="n"/>
+      <c r="O33" s="261" t="n"/>
+      <c r="P33" s="197" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="Q33" s="197" t="inlineStr">
+        <is>
+          <t>Round-off</t>
+        </is>
+      </c>
+      <c r="R33" s="197" t="n"/>
+      <c r="S33" s="261" t="n"/>
+      <c r="T33" s="197" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="U33" s="261" t="n"/>
+      <c r="V33" s="261" t="n"/>
+      <c r="W33" s="261" t="n"/>
     </row>
     <row r="34" ht="17.5" customHeight="1">
-      <c r="A34" s="171" t="n"/>
-      <c r="C34" s="171" t="n"/>
-      <c r="F34" s="169" t="n"/>
-      <c r="P34" s="180" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T34" s="181" t="inlineStr"/>
-      <c r="Y34" s="171" t="n"/>
-    </row>
-    <row r="35" ht="20.5" customHeight="1">
-      <c r="A35" s="169" t="n">
-        <v>3</v>
-      </c>
-      <c r="C35" s="171" t="inlineStr">
-        <is>
-          <t>Cước vận chuyển KCN Yên Bình - KCN Phố Nối A, Hưng Yên</t>
-        </is>
-      </c>
-      <c r="F35" s="172">
-        <f>HĐ!H17</f>
-        <v/>
-      </c>
-      <c r="I35" s="174" t="n">
-        <v>1</v>
-      </c>
-      <c r="L35" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M35" s="267">
-        <f>HĐ!B17</f>
-        <v/>
-      </c>
-      <c r="P35" s="65">
-        <f>HĐ!N17</f>
-        <v/>
-      </c>
-      <c r="Q35" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" s="268">
-        <f>P35</f>
-        <v/>
-      </c>
-      <c r="T35" s="179" t="n"/>
-      <c r="Z35" s="171" t="n"/>
-    </row>
-    <row r="36" ht="17.5" customHeight="1">
-      <c r="A36" s="171" t="inlineStr"/>
-      <c r="C36" s="171" t="n"/>
-      <c r="F36" s="169" t="n"/>
-      <c r="P36" s="180" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T36" s="181" t="inlineStr"/>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="169" t="n">
-        <v>4</v>
-      </c>
-      <c r="C37" s="171" t="inlineStr">
-        <is>
-          <t>Cước vận chuyển KCN Yên Bình - KCN Đồng Văn 3, Ninh Bình</t>
-        </is>
-      </c>
-      <c r="F37" s="172">
-        <f>HĐ!H18</f>
-        <v/>
-      </c>
-      <c r="I37" s="174" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M37" s="267">
-        <f>HĐ!B18</f>
-        <v/>
-      </c>
-      <c r="P37" s="65">
-        <f>HĐ!N18</f>
-        <v/>
-      </c>
-      <c r="Q37" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" s="268">
-        <f>P37</f>
-        <v/>
-      </c>
-      <c r="T37" s="179" t="n"/>
-    </row>
-    <row r="38" ht="17.5" customHeight="1">
-      <c r="A38" s="171" t="inlineStr"/>
-      <c r="C38" s="171" t="n"/>
-      <c r="F38" s="169" t="n"/>
-      <c r="P38" s="180" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T38" s="181" t="inlineStr"/>
-    </row>
-    <row r="39" ht="17.5" customHeight="1">
-      <c r="A39" s="169" t="n">
-        <v>5</v>
-      </c>
-      <c r="C39" s="171" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cước vận chuyển KCN Bình Xuyên- KCN Yên Bình </t>
-        </is>
-      </c>
-      <c r="F39" s="172">
-        <f>HĐ!H19</f>
-        <v/>
-      </c>
-      <c r="I39" s="174" t="n">
-        <v>1</v>
-      </c>
-      <c r="L39" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M39" s="267">
-        <f>HĐ!B19</f>
-        <v/>
-      </c>
-      <c r="P39" s="65">
-        <f>HĐ!N19</f>
-        <v/>
-      </c>
-      <c r="Q39" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" s="268">
-        <f>P39*I39</f>
-        <v/>
-      </c>
-      <c r="T39" s="179" t="n"/>
-    </row>
-    <row r="40" ht="17.5" customHeight="1">
-      <c r="A40" s="171" t="inlineStr"/>
-      <c r="C40" s="171" t="n"/>
-      <c r="F40" s="169" t="n"/>
-      <c r="P40" s="180" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T40" s="181" t="inlineStr"/>
-    </row>
-    <row r="41" ht="20.5" customHeight="1">
-      <c r="A41" s="169" t="n">
-        <v>6</v>
-      </c>
-      <c r="C41" s="171" t="inlineStr">
-        <is>
-          <t>Cước vận chuyển KCN Yên Bình - KCN Đồng Lạng, Phú Thọ</t>
-        </is>
-      </c>
-      <c r="F41" s="172">
-        <f>HĐ!H20</f>
-        <v/>
-      </c>
-      <c r="I41" s="174" t="n">
-        <v>1</v>
-      </c>
-      <c r="L41" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M41" s="267">
-        <f>HĐ!B20</f>
-        <v/>
-      </c>
-      <c r="P41" s="65">
-        <f>HĐ!N20</f>
-        <v/>
-      </c>
-      <c r="Q41" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" s="268">
-        <f>P41*I41</f>
-        <v/>
-      </c>
-      <c r="T41" s="179" t="n"/>
-    </row>
-    <row r="42" ht="17.5" customHeight="1">
-      <c r="A42" s="171" t="inlineStr"/>
-      <c r="C42" s="171" t="n"/>
-      <c r="F42" s="169" t="n"/>
-      <c r="P42" s="180" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T42" s="181" t="inlineStr"/>
-    </row>
-    <row r="43" ht="17.5" customHeight="1">
-      <c r="A43" s="169" t="n">
-        <v>7</v>
-      </c>
-      <c r="C43" s="171" t="inlineStr">
-        <is>
-          <t>Cước vận chuyển KCN Đồng Lạng, Phú Thọ- KCN Yên Bình</t>
-        </is>
-      </c>
-      <c r="F43" s="172">
-        <f>HĐ!H21</f>
-        <v/>
-      </c>
-      <c r="I43" s="174" t="n">
-        <v>1</v>
-      </c>
-      <c r="L43" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M43" s="267">
-        <f>HĐ!B21</f>
-        <v/>
-      </c>
-      <c r="P43" s="65">
-        <f>HĐ!N21</f>
-        <v/>
-      </c>
-      <c r="Q43" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="R43" s="268">
-        <f>P43*I43</f>
-        <v/>
-      </c>
-      <c r="T43" s="179" t="n"/>
-    </row>
-    <row r="44" ht="17.5" customHeight="1">
-      <c r="A44" s="171" t="inlineStr"/>
-      <c r="C44" s="171" t="n"/>
-      <c r="F44" s="169" t="n"/>
-      <c r="P44" s="180" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T44" s="181" t="inlineStr"/>
-    </row>
-    <row r="45" ht="17.5" customHeight="1">
-      <c r="A45" s="206" t="n">
-        <v>8</v>
-      </c>
-      <c r="C45" s="171" t="inlineStr">
-        <is>
-          <t>Cước vận chuyển KCN Yên Bình - KCN Bình Xuyên</t>
-        </is>
-      </c>
-      <c r="F45" s="172">
-        <f>HĐ!H22</f>
-        <v/>
-      </c>
-      <c r="I45" s="207" t="n">
-        <v>1</v>
-      </c>
-      <c r="L45" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M45" s="267">
-        <f>HĐ!B22</f>
-        <v/>
-      </c>
-      <c r="P45" s="65">
-        <f>HĐ!N22</f>
-        <v/>
-      </c>
-      <c r="Q45" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="R45" s="269">
-        <f>P45*I45</f>
-        <v/>
-      </c>
-      <c r="T45" s="209" t="n"/>
-    </row>
-    <row r="46" ht="17.5" customHeight="1">
-      <c r="A46" s="206" t="n"/>
-      <c r="C46" s="205" t="n"/>
-      <c r="F46" s="72" t="n"/>
-      <c r="G46" s="73" t="n"/>
-      <c r="H46" s="73" t="n"/>
-      <c r="I46" s="207" t="n"/>
-      <c r="L46" s="68" t="n"/>
-      <c r="M46" s="74" t="n"/>
-      <c r="P46" s="205" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T46" s="209" t="n"/>
-    </row>
-    <row r="47" ht="17.5" customHeight="1">
-      <c r="A47" s="206" t="n">
-        <v>9</v>
-      </c>
-      <c r="C47" s="171" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cước vận chuyển KCN Bình Xuyên- KCN Yên Bình </t>
-        </is>
-      </c>
-      <c r="F47" s="172">
-        <f>HĐ!H23</f>
-        <v/>
-      </c>
-      <c r="I47" s="207" t="n">
-        <v>1</v>
-      </c>
-      <c r="L47" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M47" s="267">
-        <f>HĐ!B23</f>
-        <v/>
-      </c>
-      <c r="P47" s="65">
-        <f>HĐ!N23</f>
-        <v/>
-      </c>
-      <c r="Q47" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="R47" s="269">
-        <f>P47*I47</f>
-        <v/>
-      </c>
-      <c r="T47" s="209" t="n"/>
-    </row>
-    <row r="48" ht="17.5" customHeight="1">
-      <c r="A48" s="206" t="n"/>
-      <c r="C48" s="205" t="n"/>
-      <c r="F48" s="72" t="n"/>
-      <c r="G48" s="73" t="n"/>
-      <c r="H48" s="73" t="n"/>
-      <c r="I48" s="207" t="n"/>
-      <c r="L48" s="68" t="n"/>
-      <c r="M48" s="74" t="n"/>
-      <c r="P48" s="205" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T48" s="209" t="n"/>
-    </row>
-    <row r="49" ht="22.4" customHeight="1">
-      <c r="A49" s="206" t="n">
-        <v>10</v>
-      </c>
-      <c r="C49" s="171" t="inlineStr">
-        <is>
-          <t>Cước vận chuyển KCN Yên Bình - Tây Ninh</t>
-        </is>
-      </c>
-      <c r="F49" s="172">
-        <f>HĐ!H24</f>
-        <v/>
-      </c>
-      <c r="I49" s="207" t="n">
-        <v>13</v>
-      </c>
-      <c r="L49" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M49" s="267">
-        <f>HĐ!B24</f>
-        <v/>
-      </c>
-      <c r="P49" s="65">
-        <f>HĐ!K24</f>
-        <v/>
-      </c>
-      <c r="Q49" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="R49" s="269">
-        <f>P49*I49</f>
-        <v/>
-      </c>
-      <c r="T49" s="209" t="n"/>
-    </row>
-    <row r="50" customFormat="1" s="75">
-      <c r="A50" s="206" t="n"/>
-      <c r="B50" s="170" t="n"/>
-      <c r="C50" s="205" t="n"/>
-      <c r="D50" s="170" t="n"/>
-      <c r="E50" s="170" t="n"/>
-      <c r="F50" s="72" t="n"/>
-      <c r="G50" s="73" t="n"/>
-      <c r="H50" s="73" t="n"/>
-      <c r="I50" s="207" t="n"/>
-      <c r="J50" s="170" t="n"/>
-      <c r="K50" s="170" t="n"/>
-      <c r="L50" s="68" t="n"/>
-      <c r="M50" s="74" t="n"/>
-      <c r="N50" s="170" t="n"/>
-      <c r="O50" s="170" t="n"/>
-      <c r="P50" s="205" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T50" s="209" t="n"/>
-      <c r="U50" s="170" t="n"/>
-      <c r="V50" s="170" t="n"/>
-      <c r="W50" s="170" t="n"/>
-    </row>
-    <row r="51" ht="22.4" customHeight="1">
-      <c r="A51" s="206" t="n">
-        <v>11</v>
-      </c>
-      <c r="C51" s="171" t="inlineStr">
-        <is>
-          <t>Cước vận chuyển KCN Yên Bình - Tây Ninh</t>
-        </is>
-      </c>
-      <c r="F51" s="172">
-        <f>HĐ!H25</f>
-        <v/>
-      </c>
-      <c r="I51" s="207" t="n">
-        <v>5</v>
-      </c>
-      <c r="L51" s="181" t="inlineStr">
-        <is>
-          <t>Chuyến</t>
-        </is>
-      </c>
-      <c r="M51" s="267">
-        <f>HĐ!B25</f>
-        <v/>
-      </c>
-      <c r="P51" s="65">
-        <f>HĐ!K25</f>
-        <v/>
-      </c>
-      <c r="Q51" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="R51" s="269">
-        <f>P51*I51</f>
-        <v/>
-      </c>
-      <c r="T51" s="209" t="n"/>
-    </row>
-    <row r="52" customFormat="1" s="75">
-      <c r="A52" s="206" t="n"/>
-      <c r="B52" s="170" t="n"/>
-      <c r="C52" s="205" t="n"/>
-      <c r="D52" s="170" t="n"/>
-      <c r="E52" s="170" t="n"/>
-      <c r="F52" s="72" t="n"/>
-      <c r="G52" s="73" t="n"/>
-      <c r="H52" s="73" t="n"/>
-      <c r="I52" s="207" t="n"/>
-      <c r="J52" s="170" t="n"/>
-      <c r="K52" s="170" t="n"/>
-      <c r="L52" s="68" t="n"/>
-      <c r="M52" s="74" t="n"/>
-      <c r="N52" s="170" t="n"/>
-      <c r="O52" s="170" t="n"/>
-      <c r="P52" s="205" t="inlineStr">
-        <is>
-          <t>Price unit 1.00</t>
-        </is>
-      </c>
-      <c r="T52" s="209" t="n"/>
-      <c r="U52" s="170" t="n"/>
-      <c r="V52" s="170" t="n"/>
-      <c r="W52" s="170" t="n"/>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="199" t="n"/>
-      <c r="B53" s="261" t="n"/>
-      <c r="C53" s="199" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="D53" s="261" t="n"/>
-      <c r="E53" s="261" t="n"/>
-      <c r="F53" s="199" t="inlineStr">
-        <is>
-          <t>Subtotal Amount</t>
-        </is>
-      </c>
-      <c r="G53" s="261" t="n"/>
-      <c r="H53" s="261" t="n"/>
-      <c r="I53" s="197" t="inlineStr">
-        <is>
-          <t>Discount</t>
-        </is>
-      </c>
-      <c r="J53" s="261" t="n"/>
-      <c r="K53" s="261" t="n"/>
-      <c r="L53" s="197" t="inlineStr">
-        <is>
-          <t>Charges</t>
-        </is>
-      </c>
-      <c r="M53" s="197" t="inlineStr">
-        <is>
-          <t>Sales tax</t>
-        </is>
-      </c>
-      <c r="N53" s="261" t="n"/>
-      <c r="O53" s="261" t="n"/>
-      <c r="P53" s="197" t="inlineStr">
-        <is>
-          <t>VAT</t>
-        </is>
-      </c>
-      <c r="Q53" s="197" t="inlineStr">
-        <is>
-          <t>Round-off</t>
-        </is>
-      </c>
-      <c r="R53" s="197" t="n"/>
-      <c r="S53" s="261" t="n"/>
-      <c r="T53" s="197" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="U53" s="261" t="n"/>
-      <c r="V53" s="261" t="n"/>
-      <c r="W53" s="261" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="75" t="n"/>
-      <c r="B54" s="75" t="n"/>
-      <c r="C54" s="76" t="inlineStr">
+      <c r="A34" s="75" t="n"/>
+      <c r="B34" s="75" t="n"/>
+      <c r="C34" s="76" t="inlineStr">
         <is>
           <t>VND</t>
         </is>
       </c>
-      <c r="D54" s="75" t="n"/>
-      <c r="E54" s="75" t="n"/>
-      <c r="F54" s="270">
+      <c r="D34" s="75" t="n"/>
+      <c r="E34" s="75" t="n"/>
+      <c r="F34" s="270">
         <f>R54</f>
         <v/>
       </c>
-      <c r="G54" s="254" t="n"/>
-      <c r="H54" s="254" t="n"/>
-      <c r="I54" s="76" t="n">
+      <c r="G34" s="254" t="n"/>
+      <c r="H34" s="254" t="n"/>
+      <c r="I34" s="76" t="n">
         <v>0</v>
       </c>
-      <c r="J54" s="76" t="n"/>
-      <c r="K54" s="76" t="n"/>
-      <c r="L54" s="76" t="n">
+      <c r="J34" s="76" t="n"/>
+      <c r="K34" s="76" t="n"/>
+      <c r="L34" s="76" t="n">
         <v>0</v>
       </c>
-      <c r="M54" s="76" t="n">
+      <c r="M34" s="76" t="n">
         <v>0</v>
       </c>
-      <c r="N54" s="76" t="n"/>
-      <c r="O54" s="76" t="n"/>
-      <c r="P54" s="271" t="n"/>
-      <c r="Q54" s="76" t="n">
+      <c r="N34" s="76" t="n"/>
+      <c r="O34" s="76" t="n"/>
+      <c r="P34" s="271" t="n"/>
+      <c r="Q34" s="76" t="n">
         <v>0</v>
       </c>
-      <c r="R54" s="272">
+      <c r="R34" s="272">
         <f>R31+R33+R35+R37+R39+R41+R43+R49+R45+R47+R51</f>
         <v/>
       </c>
-      <c r="S54" s="254" t="n"/>
-      <c r="T54" s="254" t="n"/>
-      <c r="U54" s="254" t="n"/>
-      <c r="V54" s="75" t="n"/>
-      <c r="W54" s="75" t="n"/>
-    </row>
-    <row r="55">
-      <c r="B55" s="78" t="inlineStr">
+      <c r="S34" s="254" t="n"/>
+      <c r="T34" s="254" t="n"/>
+      <c r="U34" s="254" t="n"/>
+      <c r="V34" s="75" t="n"/>
+      <c r="W34" s="75" t="n"/>
+    </row>
+    <row r="35" ht="20.5" customHeight="1">
+      <c r="B35" s="78" t="inlineStr">
         <is>
           <t>Other Conditions:</t>
         </is>
       </c>
-      <c r="C55" s="78" t="n"/>
-    </row>
-    <row r="56">
-      <c r="B56" s="78" t="n">
+      <c r="C35" s="78" t="n"/>
+    </row>
+    <row r="36" ht="17.5" customHeight="1">
+      <c r="B36" s="78" t="n">
         <v>1</v>
       </c>
-      <c r="C56" s="78" t="inlineStr">
+      <c r="C36" s="78" t="inlineStr">
         <is>
           <t>Purchase Condition: As mutual Purchase and Sales Agreement</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" s="78" t="n">
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="78" t="n">
         <v>2</v>
       </c>
-      <c r="C57" s="78" t="inlineStr">
+      <c r="C37" s="78" t="inlineStr">
         <is>
           <t>Inspection: As Dainese Vietnam QC team's requirement</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="78" t="n">
+    <row r="38" ht="17.5" customHeight="1">
+      <c r="B38" s="78" t="n">
         <v>3</v>
       </c>
-      <c r="C58" s="78" t="inlineStr">
+      <c r="C38" s="78" t="inlineStr">
         <is>
           <t>Packing: The Seller has responsibility to packs the goods properly and be in accordance with the Technical Specification</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" s="78" t="n">
+    <row r="39" ht="17.5" customHeight="1">
+      <c r="B39" s="78" t="n">
         <v>4</v>
       </c>
-      <c r="C59" s="78" t="inlineStr">
+      <c r="C39" s="78" t="inlineStr">
         <is>
           <t>Partial Shipment: Allowed</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="78" t="n">
+    <row r="40" ht="17.5" customHeight="1">
+      <c r="B40" s="78" t="n">
         <v>5</v>
       </c>
-      <c r="C60" s="78" t="inlineStr">
+      <c r="C40" s="78" t="inlineStr">
         <is>
           <t>The Price is VAT excluded</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="B61" s="78" t="n">
+    <row r="41" ht="20.5" customHeight="1">
+      <c r="B41" s="78" t="n">
         <v>6</v>
       </c>
-      <c r="C61" s="78" t="inlineStr">
+      <c r="C41" s="78" t="inlineStr">
         <is>
           <t>Warranty term: As mutual Purchase and Sales Agreement</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="B62" s="78" t="inlineStr">
+    <row r="42" ht="17.5" customHeight="1">
+      <c r="B42" s="78" t="inlineStr">
         <is>
           <t>Maturities due in August and at the end of December will be extended to 10th of the following month.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="B63" s="78" t="inlineStr">
+    <row r="43" ht="17.5" customHeight="1">
+      <c r="B43" s="78" t="inlineStr">
         <is>
           <t>Kindly check this order and send it back countersigned for approval.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="B64" s="78" t="inlineStr">
+    <row r="44" ht="17.5" customHeight="1">
+      <c r="B44" s="78" t="inlineStr">
         <is>
           <t>Please let us know any error and omission you might find. Without your communication within 5 days from receipt of</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="B65" s="78" t="inlineStr">
+    <row r="45" ht="17.5" customHeight="1">
+      <c r="B45" s="78" t="inlineStr">
         <is>
           <t>this order, it will be considered as accepted and confirmed in all its parts. Delivery date is of primary importance to</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="B66" s="78" t="inlineStr">
+    <row r="46" ht="17.5" customHeight="1">
+      <c r="B46" s="78" t="inlineStr">
         <is>
           <t>DAINESE Vietnam. Please always indicate the order number and date on your invoice. Thank you and Best regards</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="C67" s="79" t="inlineStr">
+    <row r="47" ht="17.5" customHeight="1">
+      <c r="C47" s="79" t="inlineStr">
         <is>
           <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ 5P VIỆT NAM</t>
         </is>
       </c>
-      <c r="Q67" s="204" t="inlineStr">
+      <c r="Q47" s="204" t="inlineStr">
         <is>
           <t>DAINESE VIETNAM</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="Q68" s="204" t="inlineStr">
+    <row r="48" ht="17.5" customHeight="1">
+      <c r="Q48" s="204" t="inlineStr">
         <is>
           <t>Purchase Office</t>
         </is>
       </c>
     </row>
+    <row r="49" ht="22.4" customHeight="1"/>
+    <row r="50" customFormat="1" s="75"/>
+    <row r="51" ht="22.4" customHeight="1"/>
+    <row r="52" customFormat="1" s="75"/>
+    <row r="53" ht="22" customHeight="1"/>
   </sheetData>
   <mergeCells count="172">
     <mergeCell ref="C44:E44"/>

</xml_diff>